<commit_message>
Add sensitivity analyses for time cut points
</commit_message>
<xml_diff>
--- a/resultados/tablas_rpsp.xlsx
+++ b/resultados/tablas_rpsp.xlsx
@@ -23,12 +23,18 @@
     <sheet name="E_IGME_ARR" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="E_DEIS_ARR" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="E_IGME_serie" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="F1_sens_descomposicion" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="F2_sens_trienios_moviles" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="F3_sens_convergencia" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="F4_sens_kitagawa" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="F5_sens_exceso" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="F6_sens_bisagra" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="212">
   <si>
     <t xml:space="preserve">serie</t>
   </si>
@@ -548,6 +554,123 @@
   <si>
     <t xml:space="preserve">valor</t>
   </si>
+  <si>
+    <t xml:space="preserve">corte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cambio_TMI_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pct_P_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cambio_P_pct_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cambio_TMI_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pct_P_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cambio_P_pct_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pct_Q_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">razon_Q4_Q1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2006-2008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2007-2009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2008-2010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2009-2011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2010-2012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2011-2013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2012-2014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2014-2016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2015-2017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2016-2018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2018-2020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2019-2021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020-2022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2021-2023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">beta_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">beta_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2011-2013 vs 2022-2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2014-2016 vs 2022-2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2016-2018 vs 2022-2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2018-2019 vs 2023-2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2019-2019 vs 2024-2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2008-2019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2012-2019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2005-2018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bisagra 2017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bisagra 2018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bisagra 2019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bisagra 2020</t>
+  </si>
 </sst>
 </file>
 
@@ -24031,6 +24154,792 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C1" t="s">
+        <v>175</v>
+      </c>
+      <c r="D1" t="s">
+        <v>176</v>
+      </c>
+      <c r="E1" t="s">
+        <v>177</v>
+      </c>
+      <c r="F1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G1" t="s">
+        <v>179</v>
+      </c>
+      <c r="H1" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-2.20550851626721</v>
+      </c>
+      <c r="C2" t="n">
+        <v>63.6485024824452</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-20.3045350875901</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-2.63962131860478</v>
+      </c>
+      <c r="F2" t="n">
+        <v>29.8297968788099</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-14.2907307113858</v>
+      </c>
+      <c r="H2" t="n">
+        <v>24.6715562228588</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-2.51621765228229</v>
+      </c>
+      <c r="C3" t="n">
+        <v>55.6693312030438</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-20.2609744729712</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-2.3289121825897</v>
+      </c>
+      <c r="F3" t="n">
+        <v>33.9388186341596</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-14.3375528091488</v>
+      </c>
+      <c r="H3" t="n">
+        <v>22.9002901225905</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-2.79258205144871</v>
+      </c>
+      <c r="C4" t="n">
+        <v>56.821179305589</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-22.9515651122077</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-2.05254778342329</v>
+      </c>
+      <c r="F4" t="n">
+        <v>29.4457829731529</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-11.3461542313392</v>
+      </c>
+      <c r="H4" t="n">
+        <v>35.1147974577139</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-3.68007466518422</v>
+      </c>
+      <c r="C5" t="n">
+        <v>56.3110088142928</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-29.9740935736255</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-1.16505516968778</v>
+      </c>
+      <c r="F5" t="n">
+        <v>10.20377870894</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-2.45552807744364</v>
+      </c>
+      <c r="H5" t="n">
+        <v>35.4491454642503</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-3.60574011231289</v>
+      </c>
+      <c r="C6" t="n">
+        <v>58.8676829820258</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-30.7020577635457</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-1.23938972255911</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5.5310416664431</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-1.43083845185554</v>
+      </c>
+      <c r="H6" t="n">
+        <v>27.5307138588055</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" t="s">
+        <v>54</v>
+      </c>
+      <c r="J1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" t="n">
+        <v>13.1303791842061</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.09534953431967</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.08951598432858</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.101570850581478</v>
+      </c>
+      <c r="F2" t="n">
+        <v>6.26274245502987</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1.61250381357796</v>
+      </c>
+      <c r="H2" t="n">
+        <v>10.9954055532878</v>
+      </c>
+      <c r="I2" t="n">
+        <v>16.739338019581</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1.52239387064497</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>182</v>
+      </c>
+      <c r="B3" t="n">
+        <v>12.8563804085321</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.0899019001215358</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.0843952987586016</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.0974697998306132</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5.73486413760401</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1.5631870948053</v>
+      </c>
+      <c r="H3" t="n">
+        <v>10.9058588555404</v>
+      </c>
+      <c r="I3" t="n">
+        <v>16.2999606433802</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1.49460586821179</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B4" t="n">
+        <v>12.5988645016132</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.0860925003874335</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.0804999882626478</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.0944383796980863</v>
+      </c>
+      <c r="F4" t="n">
+        <v>5.03423812164973</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.4918034468054</v>
+      </c>
+      <c r="H4" t="n">
+        <v>10.7243712925056</v>
+      </c>
+      <c r="I4" t="n">
+        <v>15.6478295706273</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1.45909062115019</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>184</v>
+      </c>
+      <c r="B5" t="n">
+        <v>12.1302544258886</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.0834903397469908</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.0788718816624024</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.0927751048835611</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.97815428792864</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1.50805881982126</v>
+      </c>
+      <c r="H5" t="n">
+        <v>10.3085182897559</v>
+      </c>
+      <c r="I5" t="n">
+        <v>14.9286133542745</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1.44818226389624</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>185</v>
+      </c>
+      <c r="B6" t="n">
+        <v>11.8731724067864</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.084292613610021</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.0792230416418057</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.0922317569496022</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.80836648402736</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1.50047182936343</v>
+      </c>
+      <c r="H6" t="n">
+        <v>10.0909483913493</v>
+      </c>
+      <c r="I6" t="n">
+        <v>14.5336370053675</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1.44026472455521</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>186</v>
+      </c>
+      <c r="B7" t="n">
+        <v>11.5485898383625</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.0816697234446231</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.0748765921769664</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.0890047618939686</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.36558935135253</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.46018041078487</v>
+      </c>
+      <c r="H7" t="n">
+        <v>9.8377035322765</v>
+      </c>
+      <c r="I7" t="n">
+        <v>13.9165490828462</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1.41461358712299</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>187</v>
+      </c>
+      <c r="B8" t="n">
+        <v>11.2169484714469</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.0748173909675138</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.0702686709429273</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.0837921124906321</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.05252776185104</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.43584436233538</v>
+      </c>
+      <c r="H8" t="n">
+        <v>9.65152160122172</v>
+      </c>
+      <c r="I8" t="n">
+        <v>13.3012608991954</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1.37815169967725</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>188</v>
+      </c>
+      <c r="B9" t="n">
+        <v>10.8178933469161</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.0739696220980122</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.0675165926272293</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.0821540309051553</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4.08150434351305</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1.45950534819177</v>
+      </c>
+      <c r="H9" t="n">
+        <v>9.37252933631207</v>
+      </c>
+      <c r="I9" t="n">
+        <v>12.7624854156313</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1.36169063415843</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>74</v>
+      </c>
+      <c r="B10" t="n">
+        <v>10.344973389984</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.0741973518753376</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.0685227297086455</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.0828154974876075</v>
+      </c>
+      <c r="F10" t="n">
+        <v>3.96562793867205</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1.46818390337146</v>
+      </c>
+      <c r="H10" t="n">
+        <v>8.92484520362645</v>
+      </c>
+      <c r="I10" t="n">
+        <v>12.1006514347289</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1.35583880265083</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>189</v>
+      </c>
+      <c r="B11" t="n">
+        <v>9.9940580878159</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.0763740132171868</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.0714472107807677</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.0861046372065055</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3.87441648384707</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.4745964565342</v>
+      </c>
+      <c r="H11" t="n">
+        <v>8.56639694136748</v>
+      </c>
+      <c r="I11" t="n">
+        <v>11.8639681142916</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1.38494260720047</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>190</v>
+      </c>
+      <c r="B12" t="n">
+        <v>9.59612417762971</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.0785908811363356</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.072023605869638</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.0867424019008379</v>
+      </c>
+      <c r="F12" t="n">
+        <v>3.50249258040199</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1.44132571682131</v>
+      </c>
+      <c r="H12" t="n">
+        <v>8.27051694980072</v>
+      </c>
+      <c r="I12" t="n">
+        <v>11.2582903028698</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1.36125593734997</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>191</v>
+      </c>
+      <c r="B13" t="n">
+        <v>9.32623377165162</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.0727527842802864</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.0662881490203382</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.0817247025442923</v>
+      </c>
+      <c r="F13" t="n">
+        <v>3.18088605523248</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1.40707852135307</v>
+      </c>
+      <c r="H13" t="n">
+        <v>8.11418758781204</v>
+      </c>
+      <c r="I13" t="n">
+        <v>10.8283761464194</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1.33449911395741</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" t="n">
+        <v>9.1175255062664</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.0778247247110677</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.0713705557322961</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.0882042821457642</v>
+      </c>
+      <c r="F14" t="n">
+        <v>3.14149007010858</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1.41198277689428</v>
+      </c>
+      <c r="H14" t="n">
+        <v>7.96685370044555</v>
+      </c>
+      <c r="I14" t="n">
+        <v>10.4031925141049</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1.30580940798788</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>192</v>
+      </c>
+      <c r="B15" t="n">
+        <v>8.82535330787558</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.0836508509518694</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.077338416181762</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.094185950211362</v>
+      </c>
+      <c r="F15" t="n">
+        <v>3.64647072282268</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1.51281899984072</v>
+      </c>
+      <c r="H15" t="n">
+        <v>7.55055029434349</v>
+      </c>
+      <c r="I15" t="n">
+        <v>10.3847519264446</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1.3753635856481</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>193</v>
+      </c>
+      <c r="B16" t="n">
+        <v>8.55072713232497</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.0910444204756331</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.0836233729403225</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.101766757145309</v>
+      </c>
+      <c r="F16" t="n">
+        <v>3.81948056612417</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1.56510656742782</v>
+      </c>
+      <c r="H16" t="n">
+        <v>7.24441955707808</v>
+      </c>
+      <c r="I16" t="n">
+        <v>10.209937586123</v>
+      </c>
+      <c r="J16" t="n">
+        <v>1.40935205445791</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>194</v>
+      </c>
+      <c r="B17" t="n">
+        <v>8.26437771333768</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.0915842447778452</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.0856472973988144</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.103032030757185</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3.63714944806777</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1.55474930665739</v>
+      </c>
+      <c r="H17" t="n">
+        <v>7.06403957185634</v>
+      </c>
+      <c r="I17" t="n">
+        <v>10.1236951837237</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1.43313115402939</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>195</v>
+      </c>
+      <c r="B18" t="n">
+        <v>8.12570309500142</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.0872773265157889</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.0805647545123847</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.0997122486784561</v>
+      </c>
+      <c r="F18" t="n">
+        <v>3.05605440427325</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1.4576868282711</v>
+      </c>
+      <c r="H18" t="n">
+        <v>7.10107575630646</v>
+      </c>
+      <c r="I18" t="n">
+        <v>9.75991762803547</v>
+      </c>
+      <c r="J18" t="n">
+        <v>1.3744280392119</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>76</v>
+      </c>
+      <c r="B19" t="n">
+        <v>8.2984725214274</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.0937615681576318</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.0854207057145047</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.106515512448007</v>
+      </c>
+      <c r="F19" t="n">
+        <v>3.43508349629552</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1.5143084923841</v>
+      </c>
+      <c r="H19" t="n">
+        <v>7.23624833270768</v>
+      </c>
+      <c r="I19" t="n">
+        <v>10.3704695660394</v>
+      </c>
+      <c r="J19" t="n">
+        <v>1.43312792613336</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
@@ -24186,6 +25095,935 @@
       </c>
       <c r="L4" t="n">
         <v>7.78937988754385</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1" t="s">
+        <v>197</v>
+      </c>
+      <c r="D1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E1" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-4.25549463304115</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.0202706252928803</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1.09537381591271</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.265048009631576</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-6.05415112567178</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.000382800885839331</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.90384509774456</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.133783847835376</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-5.71657740877746</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.000382387879811173</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.7998338777222</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.237939894701046</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-5.11489761552093</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.000187853483327622</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.38748807808476</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.233151706474517</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-4.15063715933559</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.000128886739561393</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.79316413321746</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.447370347949556</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E1" t="s">
+        <v>103</v>
+      </c>
+      <c r="F1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G1" t="s">
+        <v>105</v>
+      </c>
+      <c r="H1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B2" t="n">
+        <v>11.2303045407677</v>
+      </c>
+      <c r="C2" t="n">
+        <v>8.29893699993866</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-2.93136754082901</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.582275821985646</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-3.51364336281465</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-19.8636238504904</v>
+      </c>
+      <c r="H2" t="n">
+        <v>119.86362385049</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>201</v>
+      </c>
+      <c r="B3" t="n">
+        <v>9.99522216073495</v>
+      </c>
+      <c r="C3" t="n">
+        <v>8.29893699993866</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-1.6962851607963</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.527030012279137</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-2.22331517307543</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-31.0696588321111</v>
+      </c>
+      <c r="H3" t="n">
+        <v>131.069658832111</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>202</v>
+      </c>
+      <c r="B4" t="n">
+        <v>9.31050339984457</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8.29893699993866</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-1.01156639990592</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.512180371588994</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-1.52374677149491</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-50.632402542891</v>
+      </c>
+      <c r="H4" t="n">
+        <v>150.632402542891</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>203</v>
+      </c>
+      <c r="B5" t="n">
+        <v>8.99655563057135</v>
+      </c>
+      <c r="C5" t="n">
+        <v>8.23992576973286</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-0.756629860838494</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.333582790069575</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-1.09021265090807</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-44.0879758168545</v>
+      </c>
+      <c r="H5" t="n">
+        <v>144.087975816854</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>204</v>
+      </c>
+      <c r="B6" t="n">
+        <v>9.18551869800669</v>
+      </c>
+      <c r="C6" t="n">
+        <v>8.50327374829051</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-0.682244949716177</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.289387681261658</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-0.971632630977835</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-42.4169766858732</v>
+      </c>
+      <c r="H6" t="n">
+        <v>142.416976685873</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J1" t="s">
+        <v>42</v>
+      </c>
+      <c r="K1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L1" t="s">
+        <v>44</v>
+      </c>
+      <c r="M1" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" t="s">
+        <v>32</v>
+      </c>
+      <c r="O1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2"/>
+      <c r="B2" t="n">
+        <v>20107</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19842.8869244773</v>
+      </c>
+      <c r="D2" t="n">
+        <v>18968</v>
+      </c>
+      <c r="E2" t="n">
+        <v>20772.025</v>
+      </c>
+      <c r="F2" t="n">
+        <v>264.113075522695</v>
+      </c>
+      <c r="G2" t="n">
+        <v>8.26623636905557</v>
+      </c>
+      <c r="H2" t="n">
+        <v>8.15765621734578</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1.01331021421066</v>
+      </c>
+      <c r="J2" t="n">
+        <v>-665.025000000001</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1139</v>
+      </c>
+      <c r="L2" t="n">
+        <v>-3.02538659008229</v>
+      </c>
+      <c r="M2" t="s">
+        <v>19</v>
+      </c>
+      <c r="N2" t="s">
+        <v>47</v>
+      </c>
+      <c r="O2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3"/>
+      <c r="B3" t="n">
+        <v>4573</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4072.34345649451</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3804.975</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4344</v>
+      </c>
+      <c r="F3" t="n">
+        <v>500.656543505489</v>
+      </c>
+      <c r="G3" t="n">
+        <v>10.1895755717571</v>
+      </c>
+      <c r="H3" t="n">
+        <v>9.07401080343347</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1.12294064802099</v>
+      </c>
+      <c r="J3" t="n">
+        <v>229</v>
+      </c>
+      <c r="K3" t="n">
+        <v>768.025</v>
+      </c>
+      <c r="L3" t="n">
+        <v>-3.78396560384422</v>
+      </c>
+      <c r="M3" t="s">
+        <v>19</v>
+      </c>
+      <c r="N3" t="s">
+        <v>47</v>
+      </c>
+      <c r="O3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4"/>
+      <c r="B4" t="n">
+        <v>20107</v>
+      </c>
+      <c r="C4" t="n">
+        <v>19558.5761792237</v>
+      </c>
+      <c r="D4" t="n">
+        <v>18707.95</v>
+      </c>
+      <c r="E4" t="n">
+        <v>20405</v>
+      </c>
+      <c r="F4" t="n">
+        <v>548.42382077629</v>
+      </c>
+      <c r="G4" t="n">
+        <v>8.26623636905557</v>
+      </c>
+      <c r="H4" t="n">
+        <v>8.04077255381922</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1.028040068753</v>
+      </c>
+      <c r="J4" t="n">
+        <v>-298</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1399.05</v>
+      </c>
+      <c r="L4" t="n">
+        <v>-3.20798910754317</v>
+      </c>
+      <c r="M4" t="s">
+        <v>19</v>
+      </c>
+      <c r="N4" t="s">
+        <v>205</v>
+      </c>
+      <c r="O4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5"/>
+      <c r="B5" t="n">
+        <v>4573</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4044.11102212688</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3762</v>
+      </c>
+      <c r="E5" t="n">
+        <v>4326.025</v>
+      </c>
+      <c r="F5" t="n">
+        <v>528.888977873124</v>
+      </c>
+      <c r="G5" t="n">
+        <v>10.1895755717571</v>
+      </c>
+      <c r="H5" t="n">
+        <v>9.01110318839658</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1.13078003422245</v>
+      </c>
+      <c r="J5" t="n">
+        <v>246.975</v>
+      </c>
+      <c r="K5" t="n">
+        <v>811</v>
+      </c>
+      <c r="L5" t="n">
+        <v>-3.85726281351572</v>
+      </c>
+      <c r="M5" t="s">
+        <v>19</v>
+      </c>
+      <c r="N5" t="s">
+        <v>205</v>
+      </c>
+      <c r="O5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6"/>
+      <c r="B6" t="n">
+        <v>20107</v>
+      </c>
+      <c r="C6" t="n">
+        <v>19372.7593078154</v>
+      </c>
+      <c r="D6" t="n">
+        <v>18382.975</v>
+      </c>
+      <c r="E6" t="n">
+        <v>20399.025</v>
+      </c>
+      <c r="F6" t="n">
+        <v>734.240692184576</v>
+      </c>
+      <c r="G6" t="n">
+        <v>8.26623636905557</v>
+      </c>
+      <c r="H6" t="n">
+        <v>7.96438093993255</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1.03790067695149</v>
+      </c>
+      <c r="J6" t="n">
+        <v>-292.025000000001</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1724.025</v>
+      </c>
+      <c r="L6" t="n">
+        <v>-3.35979826512709</v>
+      </c>
+      <c r="M6" t="s">
+        <v>19</v>
+      </c>
+      <c r="N6" t="s">
+        <v>50</v>
+      </c>
+      <c r="O6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7"/>
+      <c r="B7" t="n">
+        <v>4573</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4015.85300724941</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3687</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4368.025</v>
+      </c>
+      <c r="F7" t="n">
+        <v>557.146992750586</v>
+      </c>
+      <c r="G7" t="n">
+        <v>10.1895755717571</v>
+      </c>
+      <c r="H7" t="n">
+        <v>8.94813857477275</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1.13873689892156</v>
+      </c>
+      <c r="J7" t="n">
+        <v>204.975</v>
+      </c>
+      <c r="K7" t="n">
+        <v>886</v>
+      </c>
+      <c r="L7" t="n">
+        <v>-3.9592568181553</v>
+      </c>
+      <c r="M7" t="s">
+        <v>19</v>
+      </c>
+      <c r="N7" t="s">
+        <v>50</v>
+      </c>
+      <c r="O7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8"/>
+      <c r="B8" t="n">
+        <v>20107</v>
+      </c>
+      <c r="C8" t="n">
+        <v>19453.9368883935</v>
+      </c>
+      <c r="D8" t="n">
+        <v>18206.925</v>
+      </c>
+      <c r="E8" t="n">
+        <v>20734.025</v>
+      </c>
+      <c r="F8" t="n">
+        <v>653.063111606483</v>
+      </c>
+      <c r="G8" t="n">
+        <v>8.26623636905557</v>
+      </c>
+      <c r="H8" t="n">
+        <v>7.9977540472547</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1.03356971472423</v>
+      </c>
+      <c r="J8" t="n">
+        <v>-627.025000000001</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1900.075</v>
+      </c>
+      <c r="L8" t="n">
+        <v>-3.27418757436559</v>
+      </c>
+      <c r="M8" t="s">
+        <v>19</v>
+      </c>
+      <c r="N8" t="s">
+        <v>206</v>
+      </c>
+      <c r="O8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9"/>
+      <c r="B9" t="n">
+        <v>4573</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4086.48320617651</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3656</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4547.025</v>
+      </c>
+      <c r="F9" t="n">
+        <v>486.516793823491</v>
+      </c>
+      <c r="G9" t="n">
+        <v>10.1895755717571</v>
+      </c>
+      <c r="H9" t="n">
+        <v>9.10551704615169</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1.11905513109369</v>
+      </c>
+      <c r="J9" t="n">
+        <v>25.9750000000004</v>
+      </c>
+      <c r="K9" t="n">
+        <v>917</v>
+      </c>
+      <c r="L9" t="n">
+        <v>-3.67216334437864</v>
+      </c>
+      <c r="M9" t="s">
+        <v>19</v>
+      </c>
+      <c r="N9" t="s">
+        <v>206</v>
+      </c>
+      <c r="O9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10"/>
+      <c r="B10" t="n">
+        <v>20107</v>
+      </c>
+      <c r="C10" t="n">
+        <v>19643.8741322018</v>
+      </c>
+      <c r="D10" t="n">
+        <v>18744.975</v>
+      </c>
+      <c r="E10" t="n">
+        <v>20591.025</v>
+      </c>
+      <c r="F10" t="n">
+        <v>463.125867798171</v>
+      </c>
+      <c r="G10" t="n">
+        <v>8.26623636905557</v>
+      </c>
+      <c r="H10" t="n">
+        <v>8.07583959719285</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1.02357609627721</v>
+      </c>
+      <c r="J10" t="n">
+        <v>-484.025000000001</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1362.025</v>
+      </c>
+      <c r="L10" t="n">
+        <v>-3.10123918687315</v>
+      </c>
+      <c r="M10" t="s">
+        <v>19</v>
+      </c>
+      <c r="N10" t="s">
+        <v>207</v>
+      </c>
+      <c r="O10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11"/>
+      <c r="B11" t="n">
+        <v>4573</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4003.88892309181</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3737.975</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4282</v>
+      </c>
+      <c r="F11" t="n">
+        <v>569.111076908188</v>
+      </c>
+      <c r="G11" t="n">
+        <v>10.1895755717571</v>
+      </c>
+      <c r="H11" t="n">
+        <v>8.92148015805053</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1.14213957675647</v>
+      </c>
+      <c r="J11" t="n">
+        <v>291</v>
+      </c>
+      <c r="K11" t="n">
+        <v>835.025</v>
+      </c>
+      <c r="L11" t="n">
+        <v>-3.90826480849937</v>
+      </c>
+      <c r="M11" t="s">
+        <v>19</v>
+      </c>
+      <c r="N11" t="s">
+        <v>207</v>
+      </c>
+      <c r="O11" t="s">
+        <v>54</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
+        <v>208</v>
+      </c>
+      <c r="C2" t="n">
+        <v>-3.12710899004003</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-2.3646198428843</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.00784021212423608</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-0.00312387971368094</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.0188043039621531</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.17904781958173</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
+        <v>209</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-3.13391752211249</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-2.08812627920637</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.010738394762439</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-0.00144510186247004</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.0229218913873481</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.102201446099172</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>210</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-3.11424840039269</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-1.80558879177638</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.0134168356317446</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-0.00105873845717944</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.0278924097206687</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.0869506742616444</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>211</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-3.12076065555942</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-1.09853178081972</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.0206588363197923</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.00311397688060067</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.0382036957589839</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.0338533518562672</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Spanish version of figures and supplementary material; harmonize sensitivity excess table with main simulation
- figuras_rpsp_es/: figures with Spanish labels (05_figuras_rpsp.R, FIG_LANG switch); layout fixes in Figures 1 and 2
- supplementary/: Material_suplementario_RPSP.pdf (Spanish) and updated English translation
- 04_analisis_rpsp.R: Table S1-E reuses the main simulation for the 2005-2019 and 2010-2019 baselines
- README and ejecutar_todo.R updated
</commit_message>
<xml_diff>
--- a/resultados/tablas_rpsp.xlsx
+++ b/resultados/tablas_rpsp.xlsx
@@ -25441,31 +25441,31 @@
         <v>20107</v>
       </c>
       <c r="C2" t="n">
-        <v>19842.8869244773</v>
+        <v>19843.7897542002</v>
       </c>
       <c r="D2" t="n">
-        <v>18968</v>
+        <v>18958</v>
       </c>
       <c r="E2" t="n">
-        <v>20772.025</v>
+        <v>20733</v>
       </c>
       <c r="F2" t="n">
-        <v>264.113075522695</v>
+        <v>263.21024579983</v>
       </c>
       <c r="G2" t="n">
         <v>8.26623636905557</v>
       </c>
       <c r="H2" t="n">
-        <v>8.15765621734578</v>
+        <v>8.1580273818104</v>
       </c>
       <c r="I2" t="n">
-        <v>1.01331021421066</v>
+        <v>1.01326411179821</v>
       </c>
       <c r="J2" t="n">
-        <v>-665.025000000001</v>
+        <v>-626</v>
       </c>
       <c r="K2" t="n">
-        <v>1139</v>
+        <v>1149</v>
       </c>
       <c r="L2" t="n">
         <v>-3.02538659008229</v>
@@ -25486,31 +25486,31 @@
         <v>4573</v>
       </c>
       <c r="C3" t="n">
-        <v>4072.34345649451</v>
+        <v>4070.31792950335</v>
       </c>
       <c r="D3" t="n">
-        <v>3804.975</v>
+        <v>3809</v>
       </c>
       <c r="E3" t="n">
-        <v>4344</v>
+        <v>4347</v>
       </c>
       <c r="F3" t="n">
-        <v>500.656543505489</v>
+        <v>502.682070496649</v>
       </c>
       <c r="G3" t="n">
         <v>10.1895755717571</v>
       </c>
       <c r="H3" t="n">
-        <v>9.07401080343347</v>
+        <v>9.06949751667443</v>
       </c>
       <c r="I3" t="n">
-        <v>1.12294064802099</v>
+        <v>1.12349946102564</v>
       </c>
       <c r="J3" t="n">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="K3" t="n">
-        <v>768.025</v>
+        <v>764</v>
       </c>
       <c r="L3" t="n">
         <v>-3.78396560384422</v>
@@ -25621,31 +25621,31 @@
         <v>20107</v>
       </c>
       <c r="C6" t="n">
-        <v>19372.7593078154</v>
+        <v>19376.8532391927</v>
       </c>
       <c r="D6" t="n">
-        <v>18382.975</v>
+        <v>18395.95</v>
       </c>
       <c r="E6" t="n">
-        <v>20399.025</v>
+        <v>20365.05</v>
       </c>
       <c r="F6" t="n">
-        <v>734.240692184576</v>
+        <v>730.146760807336</v>
       </c>
       <c r="G6" t="n">
         <v>8.26623636905557</v>
       </c>
       <c r="H6" t="n">
-        <v>7.96438093993255</v>
+        <v>7.96606400575256</v>
       </c>
       <c r="I6" t="n">
-        <v>1.03790067695149</v>
+        <v>1.03768138984149</v>
       </c>
       <c r="J6" t="n">
-        <v>-292.025000000001</v>
+        <v>-258.049999999996</v>
       </c>
       <c r="K6" t="n">
-        <v>1724.025</v>
+        <v>1711.05</v>
       </c>
       <c r="L6" t="n">
         <v>-3.35979826512709</v>

</xml_diff>